<commit_message>
docs: agregar matriz en Excel (punto 1)
</commit_message>
<xml_diff>
--- a/Book.xlsx
+++ b/Book.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2B468A8-4EEA-4C56-9DE1-80E8EB1940AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\santi\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FE275C-D84C-4FFF-84C8-A1315EC10722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="60">
   <si>
     <t>Metodo</t>
   </si>
@@ -72,9 +77,6 @@
     <t xml:space="preserve">POST </t>
   </si>
   <si>
-    <t>`/api/v1/turnos`</t>
-  </si>
-  <si>
     <t>Crear turnos</t>
   </si>
   <si>
@@ -84,31 +86,6 @@
     <t>Admin</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre nulo o vacío, teléfono que no tenga 10 dígitos o correo inválido (manejo de @gmail.com) </t>
-  </si>
-  <si>
-    <t>Disponibilidad de franja, barbero disponible</t>
-  </si>
-  <si>
-    <t>El servicio, el barbero, fecha y hora</t>
-  </si>
-  <si>
-    <t>id:a2sfasd45f6adfs,idturno:1,Especialidad:barba,descripcion:Afeitado con navaja ,timestamp:10/14/2026-1:56 03.3373</t>
-  </si>
-  <si>
-    <t>Los datos del cliente junto con los datos de entrada y una confirmacion de que el turno fue creado</t>
-  </si>
-  <si>
-    <t>cache-control: no-chache, no-store, max-age=0,must-revalidate
-content-type: application/json
-date: tue, 13 Oct 2026 16:26:32 GMT
-expires: 0
-pragma: no-cache</t>
-  </si>
-  <si>
-    <t>`/api/v1/reservas/`</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reservar un turno </t>
   </si>
   <si>
@@ -118,24 +95,9 @@
     <t xml:space="preserve">CLIENTE </t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre nulo o vacío, teléfono que no tenga 10 dígitos o correo inválido (manejo de @gmail.com),Ningún barbero con la especialidad requerida está libre en esa franja ,  Hay 3 reservas en esa fecha y hora (máx. 3 clientes por hora) o no existe turno DISPONIBLE en la franja </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disponibilidad de franja, Barbero disponible, Datos del cliente, Servicio permitido  </t>
-  </si>
-  <si>
-    <t>Datos del cliente, El servicio, el barbero, fecha y hora</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> La reserva queda CONFIRMADA, el turno OCUPADO y el total es la suma de los servicios. Sin preferencia de barbero, el sistema asigna uno disponible con la especialidad requerida.</t>
-  </si>
-  <si>
     <t>GET</t>
   </si>
   <si>
-    <t>`/api/v1/turnos/id_reservas/estado?estado=Realizada`</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ver mis turnos realizados </t>
   </si>
   <si>
@@ -145,57 +107,347 @@
     <t>CLIENTE </t>
   </si>
   <si>
-    <t>Nombre nulo o vacío, teléfono que no tenga 10 dígitos o correo inválido (manejo de @gmail.com)</t>
-  </si>
-  <si>
-    <t>Datos del cliente </t>
-  </si>
-  <si>
-    <t>Inicio de sesion, solicitud de consulta y la organizacion de fecha  y hora</t>
-  </si>
-  <si>
-    <t>las reservas del cliente autenticado; su identidad se obtiene de la sesión token, no de un identificador enviado por el cliente. Incluye todas las reservas realizadas por ese usuario, ordenadas por fecha y hora de manera descendente</t>
-  </si>
-  <si>
-    <t>`/api/v1/turnos/estado?estado=Realizada`</t>
-  </si>
-  <si>
     <t>Ver todos los turnos realizados </t>
   </si>
   <si>
     <t>ADMIN </t>
   </si>
   <si>
-    <t>Los token de las reservas de los clientes con reservas tanto pasadas como futuras</t>
-  </si>
-  <si>
-    <t>las reservas de todos los clientes, pasadas y futuras, ordenadas por fecha y hora de manera descendente.</t>
-  </si>
-  <si>
-    <t>/auth/login</t>
-  </si>
-  <si>
     <t>Iniciar Sesión </t>
   </si>
   <si>
     <t>CLIENTE  y Admin</t>
   </si>
   <si>
-    <t>Datos de inicio de sesion correctos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El usuario puede iniciar sesión para acceder a las funcionalidades que tiene permitidas, los usuarios administrador y los clientes son usuarios predefinidos que tienen que crear por medio de Base de datos, con su correo y contraseña. </t>
-  </si>
-  <si>
-    <t>Respuestas preguntas:                                                                                                                                                                                                                                                                                                                 a. la validacion de entrada verifica que los daos enviados por el musuario tengan el formato, tipo y estruvtura, la validacion de negocio comprueba que la solicitud cumpla las reglas y restriccciones de propias del Sistema
-b. La api debe responder de manera consistente indicando los errores encontrados sin crear el turno cuando la solicitud no cumple las condiciones necesarias</t>
+    <t>/api/v1/auth/login</t>
+  </si>
+  <si>
+    <t>/api/v1/turnos</t>
+  </si>
+  <si>
+    <t>/api/v1/reservas</t>
+  </si>
+  <si>
+    <t>/api/v1/reservas/mis-turnos</t>
+  </si>
+  <si>
+    <t>• correo: no nulo, no vacío, formato válido de email.
+• password: no nulo, no vacío.</t>
+  </si>
+  <si>
+    <t>1. El usuario debe existir en MongoDB (usuarios predefinidos en base de datos).
+2. La contraseña debe coincidir con el hash BCrypt registrado.
+3. El usuario debe poseer un rol activo (ROLE_ADMIN o ROLE_CLIENTE).</t>
+  </si>
+  <si>
+    <t>• correo: String (Obligatorio)
+• password: String (Obligatorio)</t>
+  </si>
+  <si>
+    <t>{
+  "correo": "admin@barber.com",
+  "password": "Password123*"
+}
+Código: 200 OK
+Significado: Autenticación exitosa. Se expide token JWT con credenciales y rol.</t>
+  </si>
+  <si>
+    <t>• token: String (Obligatorio, Bearer)
+• tipo: String (Obligatorio, "Bearer")
+• correo: String (Obligatorio)
+• rol: String (Obligatorio, ROLE_ADMIN / ROLE_CLIENTE)</t>
+  </si>
+  <si>
+    <t>Éxito:
+[200 OK]:
+{
+  "token": "eyJhbGciOiJIUzM4NCIsInR5cCI6IkpXVCJ9...",
+  "tipo": "Bearer",
+  "correo": "admin@barber.com",
+  "rol": "ROLE_ADMIN"
+}
+Errores:
+[400 Bad Request]:
+{
+  "codigo": "ERR-400",
+  "mensaje": "Correo y contraseña son obligatorios."
+}
+[401 Unauthorized]:
+{
+  "codigo": "ERR-401",
+  "mensaje": "Credenciales inválidas. Correo o contraseña incorrectos."
+}</t>
+  </si>
+  <si>
+    <t>• nombreBarbero: no nulo, no vacío.
+• fecha: formato ISO YYYY-MM-DD, no nulo.
+• horaInicio: formato HH:00 (en punto), no nulo.</t>
+  </si>
+  <si>
+    <t>1. El barbero debe existir en catálogo (Miguel, Laura o Andrés).
+2. La fecha debe ser futura (&gt; hoy).
+3. La fecha debe coincidir con un día laboral del barbero:
+   - Miguel: Lunes a Jueves
+   - Laura: Lunes a Viernes
+   - Andrés: Martes, Jueves, Sábados y Domingos
+4. La hora debe iniciar dentro de su jornada laboral:
+   - Miguel/Laura: 10:00 a 17:00
+   - Andrés: 10:00 a 14:00
+5. No duplicar barbero + fecha + horaInicio.
+6. El turno nace en estado DISPONIBLE.</t>
+  </si>
+  <si>
+    <t>• nombreBarbero: String (Obligatorio)
+• fecha: String (Obligatorio, YYYY-MM-DD)
+• horaInicio: String (Obligatorio, HH:mm)</t>
+  </si>
+  <si>
+    <t>{
+  "nombreBarbero": "Miguel",
+  "fecha": "2026-10-20",
+  "horaInicio": "10:00"
+}
+Código: 201 Created
+Significado: Turno creado y publicado exitosamente en estado DISPONIBLE.</t>
+  </si>
+  <si>
+    <t>• id: String (Obligatorio)
+• nombreBarbero: String (Obligatorio)
+• fecha: String (Obligatorio)
+• horaInicio: String (Obligatorio)
+• horaFin: String (Obligatorio, +1h)
+• estado: String (Obligatorio, "DISPONIBLE")</t>
+  </si>
+  <si>
+    <t>Éxito:
+[201 Created]:
+{
+  "id": "670c5e1f0e4b8a2134567801",
+  "nombreBarbero": "Miguel",
+  "fecha": "2026-10-20",
+  "horaInicio": "10:00",
+  "horaFin": "11:00",
+  "estado": "DISPONIBLE"
+}
+Errores:
+[400 Bad Request]:
+{"codigo": "ERR-400", "mensaje": "Formato de fecha u hora incorrecto."}
+[404 Not Found]:
+{"codigo": "ERR-404", "mensaje": "El barbero especificado no existe."}
+[409 Conflict]:
+{"codigo": "ERR-409", "mensaje": "Turno duplicado para este barbero en esa fecha y hora."}
+[422 Unprocessable]:
+{"codigo": "ERR-422", "mensaje": "Fecha no futura o fuera de horario/días del barbero."}
+[403 Forbidden]:
+{"codigo": "ERR-403", "mensaje": "Acceso denegado (requiere rol ADMIN)."}
+[401 Unauthorized]:
+{"codigo": "ERR-401", "mensaje": "Token ausente o inválido."}</t>
+  </si>
+  <si>
+    <t>• fecha: formato YYYY-MM-DD, no nulo.
+• hora: formato HH:00, no nulo.
+• nombreCliente: no nulo, no vacío ni solo espacios (E03).
+• telefonoCliente: exactamente 10 dígitos numéricos (E07).
+• correoCliente: formato válido con dominio @gmail.com (E08).
+• servicios: lista no vacía de códigos de catálogo (E09).
+• nombreBarbero: opcional.</t>
+  </si>
+  <si>
+    <t>Cadena de 5 validaciones en orden estricto:
+1. Disponibilidad de franja:
+   - Máx. 3 reservas por hora en total (E01 -&gt; 409).
+   - Existencia de turno DISPONIBLE en la franja (404/409).
+2. Barbero y especialidad:
+   - Barbero con especialidad para todos los servicios pedidos (E02 -&gt; 422).
+   - Si no se especifica barbero: asignar disponible con especialidad. Si ninguno disponible -&gt; E100 (409/422).
+3. Datos del cliente:
+   - Nombre inválido (E03 -&gt; 400).
+   - Teléfono inválido (E07 -&gt; 400).
+   - Correo inválido / dominio no gmail.com (E08 -&gt; 400).
+4. Servicio permitido:
+   - Todos deben existir en catálogo activo (E09 -&gt; 404).
+5. Confirmación:
+   - Reserva CONFIRMADA, turno OCUPADO, total = suma de servicios.</t>
+  </si>
+  <si>
+    <t>• fecha: String (Obligatorio)
+• hora: String (Obligatorio)
+• nombreCliente: String (Obligatorio)
+• telefonoCliente: String (Obligatorio, 10 dígitos)
+• correoCliente: String (Obligatorio, @gmail.com)
+• servicios: List&lt;String&gt; (Obligatorio)
+• nombreBarbero: String (Opcional)</t>
+  </si>
+  <si>
+    <t>{
+  "fecha": "2026-10-20",
+  "hora": "10:00",
+  "nombreCliente": "Carlos Mendoza",
+  "telefonoCliente": "3101234567",
+  "correoCliente": "carlos.mendoza@gmail.com",
+  "servicios": ["SER-001", "SER-004"],
+  "nombreBarbero": "Andrés"
+}
+Código: 201 Created
+Significado: Reserva confirmada, turno pasa a OCUPADO y total calculado.</t>
+  </si>
+  <si>
+    <t>• idReserva: String (Obligatorio)
+• turnoId: String (Obligatorio)
+• fecha: String (Obligatorio)
+• hora: String (Obligatorio)
+• nombreBarbero: String (Obligatorio)
+• nombreCliente: String (Obligatorio)
+• correoCliente: String (Obligatorio)
+• telefonoCliente: String (Obligatorio)
+• servicios: List&lt;Object&gt; (Obligatorio)
+• total: Double (Obligatorio)
+• estado: String (Obligatorio, "CONFIRMADA")</t>
+  </si>
+  <si>
+    <t>Éxito:
+[201 Created]:
+{
+  "idReserva": "670c5e1f0e4b8a2134567899",
+  "turnoId": "670c5e1f0e4b8a2134567801",
+  "fecha": "2026-10-20",
+  "hora": "10:00",
+  "nombreBarbero": "Andrés",
+  "nombreCliente": "Carlos Mendoza",
+  "total": 45000.0,
+  "estado": "CONFIRMADA"
+}
+Errores de negocio:
+[409 Conflict]: {"codigo": "E01", "mensaje": "Franja llena (máx 3 reservas)."}
+[422 Unprocessable]: {"codigo": "E02", "mensaje": "Especialidad incompatible."}
+[400 Bad Request]: {"codigo": "E03", "mensaje": "Nombre inválido."}
+[400 Bad Request]: {"codigo": "E07", "mensaje": "Teléfono inválido (10 dígitos)."}
+[400 Bad Request]: {"codigo": "E08", "mensaje": "Correo inválido (@gmail.com)."}
+[409 Conflict]: {"codigo": "E100", "mensaje": "Barbero no disponible."}
+[404 Not Found]: {"codigo": "E09", "mensaje": "Servicio inexistente."}
+[403 Forbidden]: {"codigo": "ERR-403", "mensaje": "Acceso denegado a ADMIN."}
+[401 Unauthorized]: {"codigo": "ERR-401", "mensaje": "Token ausente o inválido."}</t>
+  </si>
+  <si>
+    <t>• Sin cuerpo en la solicitud (GET).
+• Cabecera requerida: Authorization: Bearer &lt;token&gt;.</t>
+  </si>
+  <si>
+    <t>1. La identidad del cliente se obtiene estrictamente de la sesión/token JWT (SecurityContext), nunca de un identificador enviado por el cliente.
+2. Consulta únicamente las reservas del cliente autenticado.
+3. Ordenadas por fecha y hora de manera descendente (DESC).</t>
+  </si>
+  <si>
+    <t>• Body: N/A (Vacío)
+• Header: Authorization: Bearer &lt;JWT_CLIENTE&gt; (Obligatorio)</t>
+  </si>
+  <si>
+    <t>N/A (Petición HTTP GET sin cuerpo JSON).
+Header: Authorization: Bearer eyJhbGciOi...
+Código: 200 OK
+Significado: Lista de reservas del cliente autenticado obtenida satisfactoriamente.</t>
+  </si>
+  <si>
+    <t>List&lt;ReservaResponse&gt;:
+• idReserva: String (Obligatorio)
+• fecha: String (Obligatorio)
+• hora: String (Obligatorio)
+• nombreBarbero: String (Obligatorio)
+• servicios: List&lt;Object&gt; (Obligatorio)
+• total: Double (Obligatorio)
+• estado: String (Obligatorio, "CONFIRMADA")</t>
+  </si>
+  <si>
+    <t>Éxito:
+[200 OK]:
+[
+  {
+    "idReserva": "670c5e1f0e4b8a2134567899",
+    "fecha": "2026-10-20",
+    "hora": "10:00",
+    "nombreBarbero": "Andrés",
+    "servicios": [
+      {"codigo": "SER-001", "nombre": "Corte clásico", "precio": 25000.0},
+      {"codigo": "SER-004", "nombre": "Afeitado con navaja", "precio": 20000.0}
+    ],
+    "total": 45000.0,
+    "estado": "CONFIRMADA"
+  }
+]
+Errores:
+[400 Bad Request]:
+{"codigo": "ERR-400", "mensaje": "Parámetros de consulta inválidos."}
+[403 Forbidden]:
+{"codigo": "ERR-403", "mensaje": "Acceso denegado (requiere rol CLIENTE)."}
+[401 Unauthorized]:
+{"codigo": "ERR-401", "mensaje": "Token ausente o inválido."}</t>
+  </si>
+  <si>
+    <t>1. Consulta las reservas de todos los clientes de la barbería (tanto pasadas como futuras).
+2. Ordenadas por fecha y hora de manera descendente (DESC).</t>
+  </si>
+  <si>
+    <t>• Body: N/A (Vacío)
+• Header: Authorization: Bearer &lt;JWT_ADMIN&gt; (Obligatorio)</t>
+  </si>
+  <si>
+    <t>N/A (Petición HTTP GET sin cuerpo JSON).
+Header: Authorization: Bearer eyJhbGciOi...
+Código: 200 OK
+Significado: Lista completa de todas las reservas de la barbería obtenida exitosamente.</t>
+  </si>
+  <si>
+    <t>List&lt;ReservaAdminResponse&gt;:
+• idReserva: String (Obligatorio)
+• fecha: String (Obligatorio)
+• hora: String (Obligatorio)
+• nombreBarbero: String (Obligatorio)
+• nombreCliente: String (Obligatorio)
+• correoCliente: String (Obligatorio)
+• telefonoCliente: String (Obligatorio)
+• servicios: List&lt;Object&gt; (Obligatorio)
+• total: Double (Obligatorio)
+• estado: String (Obligatorio, "CONFIRMADA")</t>
+  </si>
+  <si>
+    <t>Éxito:
+[200 OK]:
+[
+  {
+    "idReserva": "670c5e1f0e4b8a2134567899",
+    "fecha": "2026-10-20",
+    "hora": "10:00",
+    "nombreBarbero": "Andrés",
+    "nombreCliente": "Carlos Mendoza",
+    "correoCliente": "carlos.mendoza@gmail.com",
+    "telefonoCliente": "3101234567",
+    "servicios": [
+      {"codigo": "SER-001", "nombre": "Corte clásico", "precio": 25000.0}
+    ],
+    "total": 25000.0,
+    "estado": "CONFIRMADA"
+  }
+]
+Errores:
+[400 Bad Request]:
+{"codigo": "ERR-400", "mensaje": "Parámetros de consulta inválidos."}
+[403 Forbidden]:
+{"codigo": "ERR-403", "mensaje": "Acceso denegado (requiere rol ADMIN)."}
+[401 Unauthorized]:
+{"codigo": "ERR-401", "mensaje": "Token ausente o inválido."}</t>
+  </si>
+  <si>
+    <t>Respuestas preguntas:                                                                                                                                                                                                                                                                                                                 a. La validación de entrada verifica que los datos enviados por el usuario tengan el formato, tipo y estructura correctos, como campos obligatorios, formatos de fecha o números de teléfono válidos. Se implementa generalmente en la capa Controller/DTO.
+La validación de negocio comprueba que la solicitud cumpla las reglas y restricciones propias del sistema, considerando las condiciones del negocio y el estado de la base de datos. Por ejemplo, verificar la disponibilidad del barbero, evitar turnos duplicados o comprobar el límite de reservas permitidas. Se implementa principalmente en la capa de servicios o dominio.
+b. La API debe identificar y comunicar los errores de forma consistente, deteniendo el proceso cuando una validación falla y evitando crear el turno o modificar la base de datos si la solicitud no cumple las condiciones necesarias. Para ello, puede utilizar una cadena de validaciones y un manejador global de excepciones.
+La respuesta debe incluir un código HTTP adecuado al tipo de error (por ejemplo, 400 para datos incorrectos o 409 para conflictos), junto con un cuerpo JSON estructurado que contenga el código de error específico, un mensaje explicativo y, cuando corresponda, una marca de tiempo timestamp.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,12 +479,6 @@
       <name val="Calibri"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF1A1A1A"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -242,7 +488,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -250,26 +496,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -290,9 +552,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -330,7 +592,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -436,7 +698,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -578,7 +840,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -586,8 +848,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D5:N21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="D3:N21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="25.140625" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" customWidth="1"/>
@@ -597,225 +859,293 @@
     <col min="11" max="11" width="34.42578125" customWidth="1"/>
     <col min="12" max="12" width="102.42578125" customWidth="1"/>
     <col min="13" max="13" width="28.7109375" customWidth="1"/>
-    <col min="14" max="14" width="36.7109375" customWidth="1"/>
+    <col min="14" max="14" width="50.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="4:14">
+    <row r="3" spans="4:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="4:14" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="4:14" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D5" s="1"/>
     </row>
-    <row r="7" spans="4:14">
-      <c r="D7" t="s">
+    <row r="6" spans="4:14" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="4:14" hidden="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N7" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="4:14" ht="134.25" customHeight="1">
-      <c r="D9" t="s">
+    <row r="8" spans="4:14" hidden="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+    </row>
+    <row r="9" spans="4:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="4:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+    </row>
+    <row r="11" spans="4:14" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="D11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="G11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="K9" t="s">
+      <c r="I11" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="N11" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+    </row>
+    <row r="13" spans="4:14" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="D13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="E13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="N9" s="4" t="s">
+      <c r="H13" s="8" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="4:14" ht="106.5">
-      <c r="D11" t="s">
+      <c r="I13" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="M13" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="N13" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D14" s="3"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+    </row>
+    <row r="15" spans="4:14" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="D15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="M15" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="N15" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D16" s="3"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+    </row>
+    <row r="17" spans="4:14" ht="360" x14ac:dyDescent="0.25">
+      <c r="D17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="E17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H11" t="s">
+      <c r="G17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="4:14" ht="121.5">
-      <c r="D13" t="s">
+      <c r="I17" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="J17" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="K17" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G13" t="s">
+      <c r="L17" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="M17" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="N17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J13" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="M13" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="N13" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="4:14" ht="91.5">
-      <c r="D15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G15" t="s">
-        <v>33</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="M15" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="N15" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="4:14" ht="137.25">
-      <c r="D17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" t="s">
-        <v>33</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="K17" t="s">
-        <v>47</v>
-      </c>
-      <c r="L17" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="N17" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="4:14" ht="106.5">
-      <c r="I21" s="4" t="s">
-        <v>49</v>
+    </row>
+    <row r="21" spans="4:14" ht="300" x14ac:dyDescent="0.25">
+      <c r="I21" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>